<commit_message>
refactor(arena): suffix colliding names with WallTV_V2 so the existing tab is untouched
Deploying the zone TV wall would have overwritten the components behind the
sandbox Caller_Performance tab. Renamed the local copies:
- GSquareSalesArena{Controller,Service,Wrapper}(+Test) -> *WallTV_V2(+Test)
- LWC gsquareSalesArena -> gsquareSalesArenaWallTV_V2
- GSquareSalesArenaMetric__mdt -> GSquareArenaTvMetric__mdt
- tab Caller_Performace -> Caller_Performance_WallTV_V2
References, permission set, manifest, README and the deployment workbook updated.
No component in the manifest exists in the sandbox org.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/deployment/Production_Deployment_Components.xlsx
+++ b/docs/deployment/Production_Deployment_Components.xlsx
@@ -373,27 +373,49 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Existing tab untouched</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sandbox Caller_Performance tab, gsquareSalesArena LWC, GSquareSalesArena Controller/Service/Wrapper and GSquareSalesArenaMetric__mdt are NOT in this package</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Not deployed (by design)</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Custom metadata records (none needed), Jest __tests__ folders, jsconfig.json</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:D16"/>
+  <autoFilter ref="A6:D17"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
@@ -472,7 +494,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decide on the Caller_Performace tab (see Tabs sheet)</t>
+          <t xml:space="preserve">Decide on the Caller_Performance_WallTV_V2 tab (see Tabs sheet)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -532,7 +554,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--tests GSquareSalesArenaControllerTest --tests GSquareSalesArenaServiceTest --tests GSquareSalesArenaWrapperTest --tests GSquareArenaBaselineJobTest --tests GSquareArenaBookingEventsTest</t>
+          <t xml:space="preserve">--tests GSquareSalesArenaControllerWallTV_V2Test --tests GSquareSalesArenaServiceWallTV_V2Test --tests GSquareSalesArenaWrapperWallTV_V2Test --tests GSquareArenaBaselineJobTest --tests GSquareArenaBookingEventsTest</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -701,13 +723,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="2" max="2" width="43" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="8" customWidth="1"/>
-    <col min="7" max="7" width="34" customWidth="1"/>
-    <col min="8" max="8" width="69" customWidth="1"/>
+    <col min="7" max="7" width="43" customWidth="1"/>
+    <col min="8" max="8" width="70" customWidth="1"/>
     <col min="9" max="9" width="70" customWidth="1"/>
   </cols>
   <sheetData>
@@ -764,7 +786,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaController</t>
+          <t xml:space="preserve">GSquareSalesArenaControllerWallTV_V2</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -774,7 +796,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -787,12 +809,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaControllerTest</t>
+          <t xml:space="preserve">GSquareSalesArenaControllerWallTV_V2Test</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/classes/GSquareSalesArenaController.cls</t>
+          <t xml:space="preserve">force-app/main/default/classes/GSquareSalesArenaControllerWallTV_V2.cls</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -807,7 +829,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaService</t>
+          <t xml:space="preserve">GSquareSalesArenaServiceWallTV_V2</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -817,7 +839,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -830,12 +852,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaServiceTest</t>
+          <t xml:space="preserve">GSquareSalesArenaServiceWallTV_V2Test</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/classes/GSquareSalesArenaService.cls</t>
+          <t xml:space="preserve">force-app/main/default/classes/GSquareSalesArenaServiceWallTV_V2.cls</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -850,7 +872,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaWrapper</t>
+          <t xml:space="preserve">GSquareSalesArenaWrapperWallTV_V2</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -860,7 +882,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -873,12 +895,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaWrapperTest</t>
+          <t xml:space="preserve">GSquareSalesArenaWrapperWallTV_V2Test</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/classes/GSquareSalesArenaWrapper.cls</t>
+          <t xml:space="preserve">force-app/main/default/classes/GSquareSalesArenaWrapperWallTV_V2.cls</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -979,7 +1001,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaControllerTest</t>
+          <t xml:space="preserve">GSquareSalesArenaControllerWallTV_V2Test</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -989,7 +1011,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1007,12 +1029,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/classes/GSquareSalesArenaControllerTest.cls</t>
+          <t xml:space="preserve">force-app/main/default/classes/GSquareSalesArenaControllerWallTV_V2Test.cls</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tests GSquareSalesArenaController</t>
+          <t xml:space="preserve">Tests GSquareSalesArenaControllerWallTV_V2</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1044,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaServiceTest</t>
+          <t xml:space="preserve">GSquareSalesArenaServiceWallTV_V2Test</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1032,7 +1054,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1050,12 +1072,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/classes/GSquareSalesArenaServiceTest.cls</t>
+          <t xml:space="preserve">force-app/main/default/classes/GSquareSalesArenaServiceWallTV_V2Test.cls</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tests GSquareSalesArenaService</t>
+          <t xml:space="preserve">Tests GSquareSalesArenaServiceWallTV_V2</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1087,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaWrapperTest</t>
+          <t xml:space="preserve">GSquareSalesArenaWrapperWallTV_V2Test</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1075,7 +1097,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1093,12 +1115,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/classes/GSquareSalesArenaWrapperTest.cls</t>
+          <t xml:space="preserve">force-app/main/default/classes/GSquareSalesArenaWrapperWallTV_V2Test.cls</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tests GSquareSalesArenaWrapper</t>
+          <t xml:space="preserve">Tests GSquareSalesArenaWrapperWallTV_V2</t>
         </is>
       </c>
     </row>
@@ -1353,12 +1375,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="2" max="2" width="29" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="70" customWidth="1"/>
-    <col min="7" max="7" width="51" customWidth="1"/>
+    <col min="7" max="7" width="56" customWidth="1"/>
     <col min="8" max="8" width="69" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1410,7 +1432,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">gsquareSalesArena</t>
+          <t xml:space="preserve">gsquareSalesArenaWallTV_V2</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1420,7 +1442,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1430,12 +1452,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">gsquareSalesArena.css, gsquareSalesArena.html, gsquareSalesArena.js, gsquareSalesArena.js-meta.xml</t>
+          <t xml:space="preserve">gsquareSalesArenaWallTV_V2.css, gsquareSalesArenaWallTV_V2.html, gsquareSalesArenaWallTV_V2.js, gsquareSalesArenaWallTV_V2.js-meta.xml</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/lwc/gsquareSalesArena</t>
+          <t xml:space="preserve">force-app/main/default/lwc/gsquareSalesArenaWallTV_V2</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1734,12 +1756,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="31" customWidth="1"/>
-    <col min="3" max="3" width="29" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="4" width="53" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="9" customWidth="1"/>
-    <col min="7" max="7" width="62" customWidth="1"/>
+    <col min="7" max="7" width="59" customWidth="1"/>
     <col min="8" max="8" width="70" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1829,12 +1851,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquare Sales Arena Metric</t>
+          <t xml:space="preserve">GSquare Arena TV Metric</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1844,7 +1866,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="F3" s="2">
@@ -1852,12 +1874,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Optional metric overrides. No records needed - the app works without them</t>
+          <t xml:space="preserve">Optional metric overrides for the TV wall (renamed copy of GSquareSalesArenaMetric__mdt, which stays untouched). No records needed</t>
         </is>
       </c>
     </row>
@@ -1909,9 +1931,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="31" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="51" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
     <col min="5" max="5" width="28" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="21" customWidth="1"/>
@@ -2864,7 +2886,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -2874,7 +2896,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Aggregate_Type__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Aggregate_Type__c</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2904,12 +2926,12 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Aggregate_Type__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Aggregate_Type__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -2919,7 +2941,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -2929,7 +2951,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Date_Field_API__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Date_Field_API__c</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2959,12 +2981,12 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Date_Field_API__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Date_Field_API__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -2974,7 +2996,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2984,7 +3006,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Denominator_Key__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Denominator_Key__c</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -3014,12 +3036,12 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Denominator_Key__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Denominator_Key__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3051,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -3039,7 +3061,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Display_Order__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Display_Order__c</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -3069,12 +3091,12 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Display_Order__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Display_Order__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3084,7 +3106,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3094,7 +3116,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Divisor__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Divisor__c</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -3124,12 +3146,12 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Divisor__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Divisor__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3161,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -3149,7 +3171,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Extra_Filter__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Extra_Filter__c</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -3179,12 +3201,12 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Extra_Filter__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Extra_Filter__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3216,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -3204,7 +3226,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Is_Rate__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Is_Rate__c</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -3234,12 +3256,12 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Is_Rate__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Is_Rate__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3249,7 +3271,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -3259,7 +3281,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Metric_Key__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Metric_Key__c</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -3289,12 +3311,12 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Metric_Key__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Metric_Key__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3304,7 +3326,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -3314,7 +3336,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Metric_Label__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Metric_Label__c</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -3344,12 +3366,12 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Metric_Label__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Metric_Label__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3381,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -3369,7 +3391,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Min_Volume_JSON__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Min_Volume_JSON__c</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -3399,12 +3421,12 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Min_Volume_JSON__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Min_Volume_JSON__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3414,7 +3436,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -3424,7 +3446,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Numerator_Key__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Numerator_Key__c</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -3454,12 +3476,12 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Numerator_Key__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Numerator_Key__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3469,7 +3491,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -3479,7 +3501,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Object_API__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Object_API__c</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -3509,12 +3531,12 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Object_API__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Object_API__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3546,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -3534,7 +3556,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Owner_Field_Alt__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Owner_Field_Alt__c</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -3564,12 +3586,12 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Owner_Field_Alt__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Owner_Field_Alt__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3601,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -3589,7 +3611,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Owner_Field_API__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Owner_Field_API__c</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -3619,12 +3641,12 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Owner_Field_API__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Owner_Field_API__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3634,7 +3656,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -3644,7 +3666,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Show_In_Boards__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Show_In_Boards__c</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -3674,12 +3696,12 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Show_In_Boards__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Show_In_Boards__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3711,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -3699,7 +3721,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Show_In_Funnel__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Show_In_Funnel__c</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -3729,12 +3751,12 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Show_In_Funnel__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Show_In_Funnel__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3744,7 +3766,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3754,7 +3776,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Status_Field_API__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Status_Field_API__c</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -3784,12 +3806,12 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Status_Field_API__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Status_Field_API__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3821,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3809,7 +3831,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Status_Values__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Status_Values__c</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -3839,12 +3861,12 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Status_Values__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Status_Values__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3876,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3864,7 +3886,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Unit__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Unit__c</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -3894,12 +3916,12 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Unit__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Unit__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -3909,7 +3931,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3919,7 +3941,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSquareSalesArenaMetric__mdt.Value_Field_API__c</t>
+          <t xml:space="preserve">GSquareArenaTvMetric__mdt.Value_Field_API__c</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -3949,12 +3971,12 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing - Update</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/objects/GSquareSalesArenaMetric__mdt/fields/Value_Field_API__c.field-meta.xml</t>
+          <t xml:space="preserve">force-app/main/default/objects/GSquareArenaTvMetric__mdt/fields/Value_Field_API__c.field-meta.xml</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4056,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apex class GSquareSalesArenaController; Read on GSquare_Arena_Booking__e</t>
+          <t xml:space="preserve">Apex class GSquareSalesArenaControllerWallTV_V2; Read on GSquare_Arena_Booking__e</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -4058,11 +4080,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="2" max="2" width="31" customWidth="1"/>
+    <col min="3" max="3" width="31" customWidth="1"/>
+    <col min="4" max="4" width="33" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="61" customWidth="1"/>
+    <col min="6" max="6" width="70" customWidth="1"/>
     <col min="7" max="7" width="70" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4109,17 +4131,17 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Caller_Performace</t>
+          <t xml:space="preserve">Caller_Performance_WallTV_V2</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Caller Performace</t>
+          <t xml:space="preserve">Caller Performance WallTV V2</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LWC gsquareSalesArena</t>
+          <t xml:space="preserve">LWC gsquareSalesArenaWallTV_V2</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -4129,12 +4151,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">force-app/main/default/tabs/Caller_Performace.tab-meta.xml</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CHECK: the sandbox already has a tab named Caller_Performance (correct spelling). This file is spelled Caller_Performace, so deploying it creates a SECOND tab. Decide before Production: rename the file to Caller_Performance or leave the tab out.</t>
+          <t xml:space="preserve">force-app/main/default/tabs/Caller_Performance_WallTV_V2.tab-meta.xml</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Separate tab. The existing Caller_Performance tab and its gsquareSalesArena LWC are NOT touched.</t>
         </is>
       </c>
     </row>

</xml_diff>